<commit_message>
fixed company_sources syntax error
</commit_message>
<xml_diff>
--- a/job_tracker.xlsx
+++ b/job_tracker.xlsx
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="D3" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
         </is>
       </c>
       <c r="D4" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" s="11" t="inlineStr">
         <is>
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="D5" s="15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" s="15" t="inlineStr">
         <is>
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="D6" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
@@ -1170,7 +1170,7 @@
         </is>
       </c>
       <c r="D11" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E11" s="7" t="inlineStr"/>
       <c r="F11" s="19" t="n">
@@ -1218,7 +1218,7 @@
         </is>
       </c>
       <c r="D12" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
@@ -1270,7 +1270,7 @@
         </is>
       </c>
       <c r="D13" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
@@ -1322,7 +1322,7 @@
         </is>
       </c>
       <c r="D14" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E14" s="11" t="inlineStr"/>
       <c r="F14" s="12" t="n">
@@ -1370,7 +1370,7 @@
         </is>
       </c>
       <c r="D15" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
@@ -1422,7 +1422,7 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
@@ -1474,7 +1474,7 @@
         </is>
       </c>
       <c r="D17" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
@@ -1526,7 +1526,7 @@
         </is>
       </c>
       <c r="D18" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
@@ -1578,7 +1578,7 @@
         </is>
       </c>
       <c r="D19" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
@@ -1630,7 +1630,7 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
@@ -1682,7 +1682,7 @@
         </is>
       </c>
       <c r="D21" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
@@ -1734,7 +1734,7 @@
         </is>
       </c>
       <c r="D22" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E22" s="11" t="inlineStr"/>
       <c r="F22" s="18" t="n">
@@ -1782,7 +1782,7 @@
         </is>
       </c>
       <c r="D23" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
@@ -1934,7 +1934,7 @@
         </is>
       </c>
       <c r="D26" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E26" s="11" t="inlineStr">
         <is>
@@ -1986,7 +1986,7 @@
         </is>
       </c>
       <c r="D27" s="23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E27" s="23" t="inlineStr">
         <is>
@@ -2038,7 +2038,7 @@
         </is>
       </c>
       <c r="D28" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E28" s="11" t="inlineStr"/>
       <c r="F28" s="18" t="n">
@@ -2086,7 +2086,7 @@
         </is>
       </c>
       <c r="D29" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
@@ -2138,7 +2138,7 @@
         </is>
       </c>
       <c r="D30" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E30" s="11" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
         </is>
       </c>
       <c r="D31" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
@@ -2242,7 +2242,7 @@
         </is>
       </c>
       <c r="D32" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E32" s="11" t="inlineStr">
         <is>
@@ -2294,7 +2294,7 @@
         </is>
       </c>
       <c r="D33" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E33" s="7" t="inlineStr"/>
       <c r="F33" s="19" t="n">
@@ -2342,7 +2342,7 @@
         </is>
       </c>
       <c r="D34" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E34" s="11" t="inlineStr"/>
       <c r="F34" s="12" t="n">
@@ -2390,7 +2390,7 @@
         </is>
       </c>
       <c r="D35" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
         </is>
       </c>
       <c r="D36" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E36" s="11" t="inlineStr">
         <is>
@@ -2494,7 +2494,7 @@
         </is>
       </c>
       <c r="D37" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E37" s="7" t="inlineStr"/>
       <c r="F37" s="20" t="n">
@@ -2542,7 +2542,7 @@
         </is>
       </c>
       <c r="D38" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E38" s="11" t="inlineStr">
         <is>
@@ -2594,7 +2594,7 @@
         </is>
       </c>
       <c r="D39" s="23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E39" s="23" t="inlineStr">
         <is>
@@ -2646,7 +2646,7 @@
         </is>
       </c>
       <c r="D40" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E40" s="11" t="inlineStr"/>
       <c r="F40" s="12" t="n">
@@ -2694,7 +2694,7 @@
         </is>
       </c>
       <c r="D41" s="23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E41" s="23" t="inlineStr">
         <is>
@@ -2746,7 +2746,7 @@
         </is>
       </c>
       <c r="D42" s="23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E42" s="23" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
         </is>
       </c>
       <c r="D43" s="23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E43" s="23" t="inlineStr">
         <is>
@@ -2850,7 +2850,7 @@
         </is>
       </c>
       <c r="D44" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
@@ -3258,7 +3258,7 @@
         </is>
       </c>
       <c r="D52" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E52" s="11" t="inlineStr"/>
       <c r="F52" s="12" t="n">
@@ -3306,7 +3306,7 @@
         </is>
       </c>
       <c r="D53" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
@@ -3358,7 +3358,7 @@
         </is>
       </c>
       <c r="D54" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E54" s="11" t="inlineStr">
         <is>
@@ -3410,7 +3410,7 @@
         </is>
       </c>
       <c r="D55" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
@@ -3462,7 +3462,7 @@
         </is>
       </c>
       <c r="D56" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E56" s="11" t="inlineStr"/>
       <c r="F56" s="12" t="n">
@@ -3510,7 +3510,7 @@
         </is>
       </c>
       <c r="D57" s="29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E57" s="29" t="inlineStr">
         <is>
@@ -3562,7 +3562,7 @@
         </is>
       </c>
       <c r="D58" s="29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E58" s="29" t="inlineStr">
         <is>
@@ -3614,7 +3614,7 @@
         </is>
       </c>
       <c r="D59" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E59" s="7" t="inlineStr"/>
       <c r="F59" s="8" t="n">
@@ -3662,7 +3662,7 @@
         </is>
       </c>
       <c r="D60" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E60" s="11" t="inlineStr"/>
       <c r="F60" s="21" t="n">
@@ -3710,7 +3710,7 @@
         </is>
       </c>
       <c r="D61" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
@@ -3762,7 +3762,7 @@
         </is>
       </c>
       <c r="D62" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E62" s="11" t="inlineStr">
         <is>
@@ -3814,7 +3814,7 @@
         </is>
       </c>
       <c r="D63" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E63" s="7" t="inlineStr"/>
       <c r="F63" s="8" t="n">
@@ -3862,7 +3862,7 @@
         </is>
       </c>
       <c r="D64" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E64" s="11" t="inlineStr">
         <is>
@@ -3914,7 +3914,7 @@
         </is>
       </c>
       <c r="D65" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
@@ -3966,7 +3966,7 @@
         </is>
       </c>
       <c r="D66" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E66" s="11" t="inlineStr"/>
       <c r="F66" s="12" t="n">
@@ -4014,7 +4014,7 @@
         </is>
       </c>
       <c r="D67" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
@@ -4066,7 +4066,7 @@
         </is>
       </c>
       <c r="D68" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E68" s="11" t="inlineStr">
         <is>
@@ -4118,7 +4118,7 @@
         </is>
       </c>
       <c r="D69" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
@@ -4170,7 +4170,7 @@
         </is>
       </c>
       <c r="D70" s="29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E70" s="29" t="inlineStr">
         <is>
@@ -4222,7 +4222,7 @@
         </is>
       </c>
       <c r="D71" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
@@ -4274,7 +4274,7 @@
         </is>
       </c>
       <c r="D72" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E72" s="11" t="inlineStr">
         <is>
@@ -4326,7 +4326,7 @@
         </is>
       </c>
       <c r="D73" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
@@ -4482,7 +4482,7 @@
         </is>
       </c>
       <c r="D76" s="11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E76" s="11" t="inlineStr">
         <is>
@@ -4534,7 +4534,7 @@
         </is>
       </c>
       <c r="D77" s="15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E77" s="15" t="inlineStr">
         <is>
@@ -4586,7 +4586,7 @@
         </is>
       </c>
       <c r="D78" s="11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E78" s="11" t="inlineStr">
         <is>
@@ -4638,7 +4638,7 @@
         </is>
       </c>
       <c r="D79" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E79" s="7" t="inlineStr">
         <is>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="D80" s="11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E80" s="11" t="inlineStr">
         <is>
@@ -4742,7 +4742,7 @@
         </is>
       </c>
       <c r="D81" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E81" s="7" t="inlineStr"/>
       <c r="F81" s="19" t="n">
@@ -4790,7 +4790,7 @@
         </is>
       </c>
       <c r="D82" s="29" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E82" s="29" t="inlineStr">
         <is>
@@ -4842,7 +4842,7 @@
         </is>
       </c>
       <c r="D83" s="29" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E83" s="29" t="inlineStr">
         <is>
@@ -4894,7 +4894,7 @@
         </is>
       </c>
       <c r="D84" s="11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E84" s="11" t="inlineStr">
         <is>
@@ -4946,7 +4946,7 @@
         </is>
       </c>
       <c r="D85" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E85" s="7" t="inlineStr">
         <is>
@@ -4998,7 +4998,7 @@
         </is>
       </c>
       <c r="D86" s="11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E86" s="11" t="inlineStr">
         <is>
@@ -5050,7 +5050,7 @@
         </is>
       </c>
       <c r="D87" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E87" s="7" t="inlineStr"/>
       <c r="F87" s="19" t="n">
@@ -5098,7 +5098,7 @@
         </is>
       </c>
       <c r="D88" s="11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E88" s="11" t="inlineStr">
         <is>
@@ -5150,7 +5150,7 @@
         </is>
       </c>
       <c r="D89" s="15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E89" s="15" t="inlineStr">
         <is>
@@ -5202,7 +5202,7 @@
         </is>
       </c>
       <c r="D90" s="11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E90" s="11" t="inlineStr">
         <is>
@@ -5254,7 +5254,7 @@
         </is>
       </c>
       <c r="D91" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E91" s="7" t="inlineStr">
         <is>
@@ -5306,7 +5306,7 @@
         </is>
       </c>
       <c r="D92" s="11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E92" s="11" t="inlineStr">
         <is>
@@ -5358,7 +5358,7 @@
         </is>
       </c>
       <c r="D93" s="23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E93" s="23" t="inlineStr">
         <is>
@@ -5666,7 +5666,7 @@
         </is>
       </c>
       <c r="D99" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E99" s="7" t="inlineStr"/>
       <c r="F99" s="19" t="n">
@@ -5714,7 +5714,7 @@
         </is>
       </c>
       <c r="D100" s="11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E100" s="11" t="inlineStr">
         <is>
@@ -5766,7 +5766,7 @@
         </is>
       </c>
       <c r="D101" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E101" s="7" t="inlineStr">
         <is>
@@ -5818,7 +5818,7 @@
         </is>
       </c>
       <c r="D102" s="11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E102" s="11" t="inlineStr"/>
       <c r="F102" s="18" t="n">
@@ -5866,7 +5866,7 @@
         </is>
       </c>
       <c r="D103" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E103" s="7" t="inlineStr">
         <is>
@@ -5918,7 +5918,7 @@
         </is>
       </c>
       <c r="D104" s="11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E104" s="11" t="inlineStr">
         <is>
@@ -5970,7 +5970,7 @@
         </is>
       </c>
       <c r="D105" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E105" s="7" t="inlineStr">
         <is>
@@ -6022,7 +6022,7 @@
         </is>
       </c>
       <c r="D106" s="11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E106" s="11" t="inlineStr">
         <is>
@@ -6074,7 +6074,7 @@
         </is>
       </c>
       <c r="D107" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E107" s="7" t="inlineStr">
         <is>
@@ -6126,7 +6126,7 @@
         </is>
       </c>
       <c r="D108" s="11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E108" s="11" t="inlineStr">
         <is>
@@ -6178,7 +6178,7 @@
         </is>
       </c>
       <c r="D109" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E109" s="7" t="inlineStr">
         <is>
@@ -6230,7 +6230,7 @@
         </is>
       </c>
       <c r="D110" s="11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E110" s="11" t="inlineStr">
         <is>
@@ -6282,7 +6282,7 @@
         </is>
       </c>
       <c r="D111" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E111" s="7" t="inlineStr">
         <is>
@@ -6334,7 +6334,7 @@
         </is>
       </c>
       <c r="D112" s="11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E112" s="11" t="inlineStr">
         <is>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="D113" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E113" s="7" t="inlineStr">
         <is>
@@ -6438,7 +6438,7 @@
         </is>
       </c>
       <c r="D114" s="11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E114" s="11" t="inlineStr">
         <is>
@@ -6490,7 +6490,7 @@
         </is>
       </c>
       <c r="D115" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E115" s="7" t="inlineStr"/>
       <c r="F115" s="19" t="n">
@@ -6538,7 +6538,7 @@
         </is>
       </c>
       <c r="D116" s="11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E116" s="11" t="inlineStr"/>
       <c r="F116" s="21" t="n">
@@ -6586,7 +6586,7 @@
         </is>
       </c>
       <c r="D117" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E117" s="7" t="inlineStr">
         <is>
@@ -6638,7 +6638,7 @@
         </is>
       </c>
       <c r="D118" s="11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E118" s="11" t="inlineStr">
         <is>
@@ -6690,7 +6690,7 @@
         </is>
       </c>
       <c r="D119" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E119" s="7" t="inlineStr">
         <is>
@@ -6742,7 +6742,7 @@
         </is>
       </c>
       <c r="D120" s="11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E120" s="11" t="inlineStr">
         <is>
@@ -6794,7 +6794,7 @@
         </is>
       </c>
       <c r="D121" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E121" s="7" t="inlineStr">
         <is>
@@ -6846,7 +6846,7 @@
         </is>
       </c>
       <c r="D122" s="11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E122" s="11" t="inlineStr">
         <is>
@@ -6898,7 +6898,7 @@
         </is>
       </c>
       <c r="D123" s="29" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E123" s="29" t="inlineStr">
         <is>
@@ -7314,7 +7314,7 @@
         </is>
       </c>
       <c r="D131" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E131" s="7" t="inlineStr"/>
       <c r="F131" s="19" t="n">
@@ -7362,7 +7362,7 @@
         </is>
       </c>
       <c r="D132" s="11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E132" s="11" t="inlineStr">
         <is>
@@ -7414,7 +7414,7 @@
         </is>
       </c>
       <c r="D133" s="3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E133" s="3" t="inlineStr">
         <is>
@@ -7466,7 +7466,7 @@
         </is>
       </c>
       <c r="D134" s="3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E134" s="3" t="inlineStr">
         <is>
@@ -7518,7 +7518,7 @@
         </is>
       </c>
       <c r="D135" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E135" s="7" t="inlineStr">
         <is>
@@ -7570,7 +7570,7 @@
         </is>
       </c>
       <c r="D136" s="3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E136" s="3" t="inlineStr">
         <is>
@@ -7622,7 +7622,7 @@
         </is>
       </c>
       <c r="D137" s="29" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E137" s="29" t="inlineStr">
         <is>
@@ -7674,7 +7674,7 @@
         </is>
       </c>
       <c r="D138" s="23" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E138" s="23" t="inlineStr">
         <is>
@@ -7726,7 +7726,7 @@
         </is>
       </c>
       <c r="D139" s="23" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E139" s="23" t="inlineStr">
         <is>
@@ -7778,7 +7778,7 @@
         </is>
       </c>
       <c r="D140" s="11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E140" s="11" t="inlineStr">
         <is>
@@ -7830,7 +7830,7 @@
         </is>
       </c>
       <c r="D141" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E141" s="7" t="inlineStr">
         <is>
@@ -7882,7 +7882,7 @@
         </is>
       </c>
       <c r="D142" s="11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E142" s="11" t="inlineStr">
         <is>
@@ -7934,7 +7934,7 @@
         </is>
       </c>
       <c r="D143" s="29" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E143" s="29" t="inlineStr">
         <is>
@@ -7986,7 +7986,7 @@
         </is>
       </c>
       <c r="D144" s="11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E144" s="11" t="inlineStr">
         <is>
@@ -8038,7 +8038,7 @@
         </is>
       </c>
       <c r="D145" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E145" s="7" t="inlineStr"/>
       <c r="F145" s="8" t="n">
@@ -8086,7 +8086,7 @@
         </is>
       </c>
       <c r="D146" s="29" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E146" s="29" t="inlineStr">
         <is>
@@ -8138,7 +8138,7 @@
         </is>
       </c>
       <c r="D147" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E147" s="7" t="inlineStr"/>
       <c r="F147" s="19" t="n">
@@ -8330,7 +8330,7 @@
         </is>
       </c>
       <c r="D151" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E151" s="7" t="inlineStr">
         <is>
@@ -8382,7 +8382,7 @@
         </is>
       </c>
       <c r="D152" s="11" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E152" s="11" t="inlineStr"/>
       <c r="F152" s="12" t="n">
@@ -8430,7 +8430,7 @@
         </is>
       </c>
       <c r="D153" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E153" s="7" t="inlineStr"/>
       <c r="F153" s="19" t="n">
@@ -8478,7 +8478,7 @@
         </is>
       </c>
       <c r="D154" s="11" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E154" s="11" t="inlineStr"/>
       <c r="F154" s="12" t="n">
@@ -8526,7 +8526,7 @@
         </is>
       </c>
       <c r="D155" s="23" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E155" s="23" t="inlineStr">
         <is>
@@ -8578,7 +8578,7 @@
         </is>
       </c>
       <c r="D156" s="23" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E156" s="23" t="inlineStr">
         <is>
@@ -8630,7 +8630,7 @@
         </is>
       </c>
       <c r="D157" s="23" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E157" s="23" t="inlineStr">
         <is>
@@ -8682,7 +8682,7 @@
         </is>
       </c>
       <c r="D158" s="11" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E158" s="11" t="inlineStr">
         <is>
@@ -8734,7 +8734,7 @@
         </is>
       </c>
       <c r="D159" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E159" s="7" t="inlineStr"/>
       <c r="F159" s="19" t="n">
@@ -8782,7 +8782,7 @@
         </is>
       </c>
       <c r="D160" s="11" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E160" s="11" t="inlineStr">
         <is>
@@ -8834,7 +8834,7 @@
         </is>
       </c>
       <c r="D161" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E161" s="7" t="inlineStr">
         <is>
@@ -8886,7 +8886,7 @@
         </is>
       </c>
       <c r="D162" s="11" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E162" s="11" t="inlineStr">
         <is>
@@ -8938,7 +8938,7 @@
         </is>
       </c>
       <c r="D163" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E163" s="7" t="inlineStr">
         <is>
@@ -9246,7 +9246,7 @@
         </is>
       </c>
       <c r="D169" s="7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E169" s="7" t="inlineStr">
         <is>
@@ -9298,7 +9298,7 @@
         </is>
       </c>
       <c r="D170" s="11" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E170" s="11" t="inlineStr">
         <is>
@@ -9350,7 +9350,7 @@
         </is>
       </c>
       <c r="D171" s="7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E171" s="7" t="inlineStr">
         <is>
@@ -9402,7 +9402,7 @@
         </is>
       </c>
       <c r="D172" s="11" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E172" s="11" t="inlineStr"/>
       <c r="F172" s="21" t="n">
@@ -9450,7 +9450,7 @@
         </is>
       </c>
       <c r="D173" s="7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E173" s="7" t="inlineStr">
         <is>
@@ -9502,7 +9502,7 @@
         </is>
       </c>
       <c r="D174" s="11" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E174" s="11" t="inlineStr">
         <is>
@@ -9554,7 +9554,7 @@
         </is>
       </c>
       <c r="D175" s="7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E175" s="7" t="inlineStr">
         <is>
@@ -9910,7 +9910,7 @@
         </is>
       </c>
       <c r="D182" s="23" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E182" s="23" t="inlineStr">
         <is>
@@ -9962,7 +9962,7 @@
         </is>
       </c>
       <c r="D183" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E183" s="7" t="inlineStr">
         <is>
@@ -10014,7 +10014,7 @@
         </is>
       </c>
       <c r="D184" s="11" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E184" s="11" t="inlineStr">
         <is>
@@ -10066,7 +10066,7 @@
         </is>
       </c>
       <c r="D185" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E185" s="7" t="inlineStr">
         <is>
@@ -10118,7 +10118,7 @@
         </is>
       </c>
       <c r="D186" s="11" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E186" s="11" t="inlineStr">
         <is>
@@ -10170,7 +10170,7 @@
         </is>
       </c>
       <c r="D187" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E187" s="7" t="inlineStr">
         <is>
@@ -10222,7 +10222,7 @@
         </is>
       </c>
       <c r="D188" s="11" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E188" s="11" t="inlineStr"/>
       <c r="F188" s="12" t="n">
@@ -10270,7 +10270,7 @@
         </is>
       </c>
       <c r="D189" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E189" s="7" t="inlineStr">
         <is>
@@ -10322,7 +10322,7 @@
         </is>
       </c>
       <c r="D190" s="11" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E190" s="11" t="inlineStr">
         <is>
@@ -10374,7 +10374,7 @@
         </is>
       </c>
       <c r="D191" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E191" s="7" t="inlineStr">
         <is>
@@ -10426,7 +10426,7 @@
         </is>
       </c>
       <c r="D192" s="11" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E192" s="11" t="inlineStr">
         <is>
@@ -10682,7 +10682,7 @@
         </is>
       </c>
       <c r="D197" s="7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E197" s="7" t="inlineStr">
         <is>
@@ -10734,7 +10734,7 @@
         </is>
       </c>
       <c r="D198" s="11" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E198" s="11" t="inlineStr">
         <is>
@@ -10786,7 +10786,7 @@
         </is>
       </c>
       <c r="D199" s="7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E199" s="7" t="inlineStr">
         <is>
@@ -10838,7 +10838,7 @@
         </is>
       </c>
       <c r="D200" s="11" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E200" s="11" t="inlineStr">
         <is>
@@ -10890,7 +10890,7 @@
         </is>
       </c>
       <c r="D201" s="7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E201" s="7" t="inlineStr">
         <is>
@@ -10942,7 +10942,7 @@
         </is>
       </c>
       <c r="D202" s="11" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E202" s="11" t="inlineStr"/>
       <c r="F202" s="18" t="n">
@@ -10990,7 +10990,7 @@
         </is>
       </c>
       <c r="D203" s="7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E203" s="7" t="inlineStr">
         <is>
@@ -11042,7 +11042,7 @@
         </is>
       </c>
       <c r="D204" s="11" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E204" s="11" t="inlineStr">
         <is>
@@ -11094,7 +11094,7 @@
         </is>
       </c>
       <c r="D205" s="7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E205" s="7" t="inlineStr">
         <is>
@@ -11146,7 +11146,7 @@
         </is>
       </c>
       <c r="D206" s="11" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E206" s="11" t="inlineStr"/>
       <c r="F206" s="12" t="n">
@@ -11194,7 +11194,7 @@
         </is>
       </c>
       <c r="D207" s="15" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E207" s="15" t="inlineStr">
         <is>
@@ -11246,7 +11246,7 @@
         </is>
       </c>
       <c r="D208" s="11" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E208" s="11" t="inlineStr">
         <is>
@@ -11298,7 +11298,7 @@
         </is>
       </c>
       <c r="D209" s="7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E209" s="7" t="inlineStr">
         <is>
@@ -11350,7 +11350,7 @@
         </is>
       </c>
       <c r="D210" s="11" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E210" s="11" t="inlineStr">
         <is>
@@ -11402,7 +11402,7 @@
         </is>
       </c>
       <c r="D211" s="7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E211" s="7" t="inlineStr">
         <is>

</xml_diff>